<commit_message>
hapus kolom status pada tabel dosen
</commit_message>
<xml_diff>
--- a/data_dosen_baru.xlsx
+++ b/data_dosen_baru.xlsx
@@ -462,11 +462,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1124097756</v>
+        <v>1176365400</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Drs. Jefri Sinaga, S.E.I</t>
+          <t>Drs. Kalim Firmansyah, S.E.I</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -476,12 +476,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>jefri0@kampus.ac.id</t>
+          <t>kalim0@kampus.ac.id</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -492,16 +492,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3294055801</v>
+        <v>2903519028</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ir. Dr. Unjani Mustofa, S.E.</t>
+          <t>drg. Irwan Zulkarnain, M.Pd</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>dr.1@kampus.ac.id</t>
+          <t>irwan1@kampus.ac.id</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -522,26 +522,26 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5568745084</v>
+        <v>8151631707</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cut Drs. Fitriani Wahyuni, S.E.</t>
+          <t>R.M. Leo Tampubolon, S.I.Kom</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>drs.2@kampus.ac.id</t>
+          <t>leo2@kampus.ac.id</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -552,11 +552,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1598242315</v>
+        <v>8548183702</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Drs. Dr. Cindy Usamah, S.Sos</t>
+          <t>Dr. Lasmanto Sinaga, S.E.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -566,12 +566,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>dr.3@kampus.ac.id</t>
+          <t>lasmanto3@kampus.ac.id</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -582,11 +582,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>8654295285</v>
+        <v>3684336417</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cut Diana Nuraini, M.Farm</t>
+          <t>R. Calista Handayani, S.T.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -596,42 +596,42 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>diana4@kampus.ac.id</t>
+          <t>calista4@kampus.ac.id</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aktif</t>
+          <t>Pensiun</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1970447586</v>
+        <v>2343431587</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>T. Drs. Mahfud Utama, S.E.I, S.H.</t>
+          <t>Dr. Ira Rahimah, S.Gz</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>drs.5@kampus.ac.id</t>
+          <t>ira5@kampus.ac.id</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -642,26 +642,26 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9285849039</v>
+        <v>7881173549</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dr. Nyana Anggraini, S.I.Kom</t>
+          <t>Dr. Janet Yuliarti, S.I.Kom</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>nyana6@kampus.ac.id</t>
+          <t>janet6@kampus.ac.id</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -672,26 +672,26 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9126681032</v>
+        <v>412481156</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Drs. Hasta Waluyo, S.T.</t>
+          <t>Ir. Aurora Nuraini, M.Farm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>hasta7@kampus.ac.id</t>
+          <t>aurora7@kampus.ac.id</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -702,11 +702,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2862998064</v>
+        <v>6467171909</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>R.M. Salsabila Anggriawan, M.M.</t>
+          <t>Dt. Anggabaya Januar, M.Ak</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Lektor</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>salsabila8@kampus.ac.id</t>
+          <t>anggabaya8@kampus.ac.id</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -732,16 +732,16 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>887360992</v>
+        <v>3267605975</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>drg. Elvin Kuswoyo, S.Kom</t>
+          <t>Cut Salimah Lestari, M.M.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>elvin9@kampus.ac.id</t>
+          <t>salimah9@kampus.ac.id</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -762,11 +762,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>347366544</v>
+        <v>9347048388</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cut Drs. Farhunnisa Marbun, S.Farm, S.Kom</t>
+          <t>dr. Indah Andriani, M.Kom.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -776,12 +776,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>drs.10@kampus.ac.id</t>
+          <t>indah10@kampus.ac.id</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -792,16 +792,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1441614365</v>
+        <v>7503867422</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>R. Cahyo Wasita, S.E., M.Pd</t>
+          <t>Ir. Lintang Novitasari, S.Pd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>cahyo11@kampus.ac.id</t>
+          <t>lintang11@kampus.ac.id</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -822,16 +822,16 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>4729660131</v>
+        <v>3811718465</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Drs. Citra Yulianti, S.E.I</t>
+          <t>R. Raharja Rajata, S.Pt</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -841,22 +841,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>citra12@kampus.ac.id</t>
+          <t>raharja12@kampus.ac.id</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Pensiun</t>
+          <t>Aktif</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5546761189</v>
+        <v>8506706152</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Puti T. Jayadi Wahyuni, S.E., S.Gz</t>
+          <t>Tgk. Intan Andriani, S.Sos</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>t.13@kampus.ac.id</t>
+          <t>intan13@kampus.ac.id</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -882,11 +882,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3582131633</v>
+        <v>7546342110</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>R.M. Laras Nashiruddin, M.Farm</t>
+          <t>Drs. Ikin Simbolon, M.TI.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -896,12 +896,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>laras14@kampus.ac.id</t>
+          <t>ikin14@kampus.ac.id</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -912,16 +912,16 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>6342976369</v>
+        <v>1679452594</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Puti Rafi Wastuti, S.E.I</t>
+          <t>Drs. Mustofa Thamrin, S.Kom</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>rafi15@kampus.ac.id</t>
+          <t>mustofa15@kampus.ac.id</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -942,11 +942,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3739261852</v>
+        <v>1658842983</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tgk. Marsudi Hutasoit, S.Farm</t>
+          <t>drg. Warsita Jailani, S.E.I</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>marsudi16@kampus.ac.id</t>
+          <t>warsita16@kampus.ac.id</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -972,11 +972,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2962893581</v>
+        <v>3491979274</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hj. Dr. Asmianto Wijayanti, M.Kom.</t>
+          <t>Cut Wirda Lailasari, M.M.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>dr.17@kampus.ac.id</t>
+          <t>wirda17@kampus.ac.id</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1002,26 +1002,26 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>4196233158</v>
+        <v>535710222</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dt. Banawi Gunarto, M.Farm</t>
+          <t>R. Hesti Prastuti, S.Gz</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>banawi18@kampus.ac.id</t>
+          <t>hesti18@kampus.ac.id</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1032,26 +1032,26 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>8730605423</v>
+        <v>242635987</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Drs. Suci Palastri, S.Ked, S.Pd</t>
+          <t>Drs. Keisha Mulyani, M.TI.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>suci19@kampus.ac.id</t>
+          <t>keisha19@kampus.ac.id</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1062,16 +1062,16 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1022825180</v>
+        <v>557092877</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>R. R.A. Ophelia Prabowo, S.Pd</t>
+          <t>Drs. Yahya Prakasa, M.M.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>r.a.20@kampus.ac.id</t>
+          <t>yahya20@kampus.ac.id</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1092,16 +1092,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1707103847</v>
+        <v>5571476047</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tgk. Puti Novi Sudiati, S.E., M.Kom.</t>
+          <t>drg. Safina Rahmawati, S.Pt</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>puti21@kampus.ac.id</t>
+          <t>safina21@kampus.ac.id</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1122,11 +1122,11 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2396883726</v>
+        <v>4714817780</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dt. Kurnia Yulianti, M.TI., S.Farm</t>
+          <t>H. Uda Dongoran, S.E.I</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1136,12 +1136,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>kurnia22@kampus.ac.id</t>
+          <t>uda22@kampus.ac.id</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1152,16 +1152,16 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>8639301362</v>
+        <v>1733473774</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dr. Syahrini Padmasari, M.M.</t>
+          <t>Dr. Mursita Jailani, S.Pt</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1171,27 +1171,27 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>syahrini23@kampus.ac.id</t>
+          <t>mursita23@kampus.ac.id</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Aktif</t>
+          <t>Pensiun</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>5278538875</v>
+        <v>9556559774</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ir. Edi Handayani, S.IP, M.Kom.</t>
+          <t>Tgk. Rudi Siregar, S.Farm</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>edi24@kampus.ac.id</t>
+          <t>rudi24@kampus.ac.id</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1212,11 +1212,11 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3786430089</v>
+        <v>6698459493</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ir. Balangga Wahyuni, M.Pd</t>
+          <t>drg. Padma Melani, S.Gz</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1226,27 +1226,27 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>balangga25@kampus.ac.id</t>
+          <t>padma25@kampus.ac.id</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Pensiun</t>
+          <t>Aktif</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>5027678490</v>
+        <v>7244794076</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dr. dr. Azalea Kusmawati, S.Sos</t>
+          <t>drg. Yahya Hutagalung, S.Psi</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Asisten Ahli</t>
+          <t>Profesor</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>dr.26@kampus.ac.id</t>
+          <t>yahya26@kampus.ac.id</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1272,26 +1272,26 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>5338883162</v>
+        <v>3202475623</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hj. Gatot Purwanti, S.Pd</t>
+          <t>R.M. Pandu Prakasa, S.T.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Lektor Kepala</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>gatot27@kampus.ac.id</t>
+          <t>pandu27@kampus.ac.id</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1302,41 +1302,41 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>961895354</v>
+        <v>8645892971</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Hj. Hasna Yuniar, S.Sos</t>
+          <t>Tgk. Teddy Gunawan, S.E.I</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Lektor Kepala</t>
+          <t>Lektor</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>hasna28@kampus.ac.id</t>
+          <t>teddy28@kampus.ac.id</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aktif</t>
+          <t>Pensiun</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>237263694</v>
+        <v>9030824756</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dr. Ilsa Uyainah, S.Psi</t>
+          <t>R.M. Dasa Megantara, M.Ak</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1346,12 +1346,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Profesor</t>
+          <t>Asisten Ahli</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ilsa29@kampus.ac.id</t>
+          <t>dasa29@kampus.ac.id</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">

</xml_diff>